<commit_message>
Comparar AMD e Apple Silicon em IA local
</commit_message>
<xml_diff>
--- a/03-Hardware/Catalogo-NVIDIA-IA-local.xlsx
+++ b/03-Hardware/Catalogo-NVIDIA-IA-local.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU_Catalogo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modelo_vs_GPU" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metricas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GPU_Catalogo'!$A$1:$L$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GPU_Catalogo'!$A$1:$Q$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Metricas'!$A$1:$L$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -426,21 +428,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="37" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="52" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="47" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,6 +511,31 @@
           <t>Piso FP16 GB</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Fabricante</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo_de_dado</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Potência_confirmada</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Tokens_s_medido</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Fonte_de_desempenho</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -556,6 +588,26 @@
       <c r="L2" t="n">
         <v>16</v>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -608,6 +660,26 @@
       <c r="L3" t="n">
         <v>16</v>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -660,6 +732,26 @@
       <c r="L4" t="n">
         <v>16</v>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -712,6 +804,26 @@
       <c r="L5" t="n">
         <v>16</v>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -764,6 +876,26 @@
       <c r="L6" t="n">
         <v>16</v>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -816,6 +948,26 @@
       <c r="L7" t="n">
         <v>16</v>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -868,6 +1020,26 @@
       <c r="L8" t="n">
         <v>16</v>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -920,6 +1092,26 @@
       <c r="L9" t="n">
         <v>16</v>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -972,6 +1164,26 @@
       <c r="L10" t="n">
         <v>16</v>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1024,6 +1236,26 @@
       <c r="L11" t="n">
         <v>16</v>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1076,6 +1308,26 @@
       <c r="L12" t="n">
         <v>16</v>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1128,6 +1380,26 @@
       <c r="L13" t="n">
         <v>16</v>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1180,6 +1452,26 @@
       <c r="L14" t="n">
         <v>16</v>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1232,6 +1524,26 @@
       <c r="L15" t="n">
         <v>16</v>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1284,6 +1596,26 @@
       <c r="L16" t="n">
         <v>16</v>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1336,6 +1668,26 @@
       <c r="L17" t="n">
         <v>16</v>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1388,6 +1740,26 @@
       <c r="L18" t="n">
         <v>16</v>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1442,9 +1814,500 @@
       <c r="L19" t="n">
         <v>16</v>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>official/secondary specs; no universal tok/s</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AMD Radeon RX 7900 XTX</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RDNA 3</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>24 GB GDDR6</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>960 GB/s</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>355</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>ROCm/Vulkan; 24 GB</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>8B/14B; 27B Q4; 70B with multi-GPU/offload</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>AMD official / ROCm status varies</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>official spec; runtime compatibility conditional</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AMD Radeon RX 7900 XT</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>RDNA 3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>20 GB GDDR6</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>800 GB/s</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>315</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ROCm/Vulkan; 20 GB</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>8B/14B; 27B Q4 with limited context</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>AMD/secondary spec</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>verify exact ROCm support before purchase</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AMD Radeon RX 7800 XT</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RDNA 3</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>16 GB GDDR6</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>624 GB/s</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>263</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ROCm/Vulkan; 16 GB</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>8B/14B; 27B Q4 tight</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>AMD/secondary spec</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>better capacity than 12GB cards, weaker software path</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AMD Radeon RX 9070 XT</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RDNA 4</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>16 GB GDDR6</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>640 GB/s</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>304</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ROCm/Vulkan; support depends on ROCm version</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>8B/14B; 27B Q4 tight</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>AMD product family / verify matrix</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>include only after ROCm matrix confirms target OS/kernel</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AMD Radeon PRO W7900</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RDNA 3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>48 GB GDDR6 ECC</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>864 GB/s</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>295</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ROCm/Vulkan; professional ECC</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>8B–70B Q4 with context dimensioned</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>AMD official</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>strong capacity, weaker ecosystem consistency than CUDA</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Apple M4 Max 40-core GPU / 128GB</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Apple Silicon UMA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>128 GB unified</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>546 GB/s</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Metal/MLX/MPS; shared CPU/GPU memory</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>8B–70B depending on quantization/context; nearly 200B claim is capacity, not speed</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Apple official</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>no official chip TDP or tokens/s in source</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Apple M4 Max 40-core GPU / 64GB</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Apple Silicon UMA</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>64 GB unified</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>546 GB/s</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Metal/MLX/MPS; shared CPU/GPU memory</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>8B–70B Q4 with context dimensioned</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Apple official</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>no official chip TDP or tokens/s in source</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Apple M4 Ultra</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Não confirmado</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Não confirmado</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Não confirmado</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Não incluir como produto lançado</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Não há ficha oficial encontrada</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Apple search status</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>do not use for purchase sizing until official announcement</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>[[03-Hardware/Referencias-de-desempenho-GPU]]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L19"/>
+  <autoFilter ref="A1:Q27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1620,4 +2483,1229 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Fabricante</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>VRAM_GB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Banda_GB_s</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Potencia_W</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fonte_dado</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Modelo_referencia</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Peso_Q4_GB</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Teto_teorico_tok_s_8B_Q4</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Teto_teorico_tok_s_por_W</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Tokens_s_medido</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RTX 3060 12GB</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" t="n">
+        <v>360</v>
+      </c>
+      <c r="E2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I2" t="n">
+        <v>90</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.5294117647058824</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RTX 3060 Ti</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>448</v>
+      </c>
+      <c r="E3" t="n">
+        <v>200</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" t="n">
+        <v>112</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RTX 4060 Ti 16GB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D4" t="n">
+        <v>288</v>
+      </c>
+      <c r="E4" t="n">
+        <v>165</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>72</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.4363636363636363</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RTX 4070 Super</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" t="n">
+        <v>504</v>
+      </c>
+      <c r="E5" t="n">
+        <v>220</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>126</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.5727272727272728</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RTX 4070 Ti Super</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D6" t="n">
+        <v>672</v>
+      </c>
+      <c r="E6" t="n">
+        <v>285</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>168</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.5894736842105263</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RTX 4080 Super</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>16</v>
+      </c>
+      <c r="D7" t="n">
+        <v>736</v>
+      </c>
+      <c r="E7" t="n">
+        <v>320</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" t="n">
+        <v>184</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RTX 4090</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>24</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1008</v>
+      </c>
+      <c r="E8" t="n">
+        <v>450</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" t="n">
+        <v>252</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RTX 3090</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24</v>
+      </c>
+      <c r="D9" t="n">
+        <v>936</v>
+      </c>
+      <c r="E9" t="n">
+        <v>350</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" t="n">
+        <v>234</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.6685714285714286</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RTX 3090 Ti</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1008</v>
+      </c>
+      <c r="E10" t="n">
+        <v>450</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>252</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RTX 5080</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D11" t="n">
+        <v>960</v>
+      </c>
+      <c r="E11" t="n">
+        <v>360</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" t="n">
+        <v>240</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RTX 5090</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>32</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1792</v>
+      </c>
+      <c r="E12" t="n">
+        <v>575</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>4</v>
+      </c>
+      <c r="I12" t="n">
+        <v>448</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.7791304347826087</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RTX 5000 Ada</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>32</v>
+      </c>
+      <c r="D13" t="n">
+        <v>576</v>
+      </c>
+      <c r="E13" t="n">
+        <v>250</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>4</v>
+      </c>
+      <c r="I13" t="n">
+        <v>144</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RTX 6000 Ada</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>48</v>
+      </c>
+      <c r="D14" t="n">
+        <v>960</v>
+      </c>
+      <c r="E14" t="n">
+        <v>300</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>240</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RTX A6000</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>48</v>
+      </c>
+      <c r="D15" t="n">
+        <v>768</v>
+      </c>
+      <c r="E15" t="n">
+        <v>300</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" t="n">
+        <v>192</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RTX PRO 6000 Blackwell</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>96</v>
+      </c>
+      <c r="E16" t="n">
+        <v>600</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>A100 80GB</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>80</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1935</v>
+      </c>
+      <c r="E17" t="n">
+        <v>300</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>483.75</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1.6125</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>H100 80GB</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>80</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3350</v>
+      </c>
+      <c r="E18" t="n">
+        <v>700</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>4</v>
+      </c>
+      <c r="I18" t="n">
+        <v>837.5</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1.196428571428571</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>H200 141GB</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>141</v>
+      </c>
+      <c r="D19" t="n">
+        <v>4800</v>
+      </c>
+      <c r="E19" t="n">
+        <v>700</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>4</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1.714285714285714</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AMD Radeon RX 7900 XTX</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>24</v>
+      </c>
+      <c r="D20" t="n">
+        <v>960</v>
+      </c>
+      <c r="E20" t="n">
+        <v>355</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>4</v>
+      </c>
+      <c r="I20" t="n">
+        <v>240</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.676056338028169</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AMD Radeon RX 7900 XT</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" t="n">
+        <v>800</v>
+      </c>
+      <c r="E21" t="n">
+        <v>315</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" t="n">
+        <v>200</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.6349206349206349</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AMD Radeon RX 7800 XT</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>16</v>
+      </c>
+      <c r="D22" t="n">
+        <v>624</v>
+      </c>
+      <c r="E22" t="n">
+        <v>263</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>4</v>
+      </c>
+      <c r="I22" t="n">
+        <v>156</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.5931558935361216</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AMD Radeon RX 9070 XT</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>16</v>
+      </c>
+      <c r="D23" t="n">
+        <v>640</v>
+      </c>
+      <c r="E23" t="n">
+        <v>304</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>4</v>
+      </c>
+      <c r="I23" t="n">
+        <v>160</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.5263157894736842</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AMD Radeon PRO W7900</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>48</v>
+      </c>
+      <c r="D24" t="n">
+        <v>864</v>
+      </c>
+      <c r="E24" t="n">
+        <v>295</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>4</v>
+      </c>
+      <c r="I24" t="n">
+        <v>216</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.7322033898305085</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>teto teórico de banda; não é benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Apple M4 Max 40-core GPU / 128GB</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>128</v>
+      </c>
+      <c r="D25" t="n">
+        <v>546</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>4</v>
+      </c>
+      <c r="I25" t="n">
+        <v>136.5</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>sem TDP oficial na fonte; tokens/s/W não calculado</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Apple M4 Max 40-core GPU / 64GB</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>64</v>
+      </c>
+      <c r="D26" t="n">
+        <v>546</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>4</v>
+      </c>
+      <c r="I26" t="n">
+        <v>136.5</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>sem TDP oficial na fonte; tokens/s/W não calculado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Apple M4 Ultra</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>official/secondary</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>8B Q4</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>4</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>sem TDP oficial na fonte; tokens/s/W não calculado</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L27"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Comparar formatos FP8 e FP4
</commit_message>
<xml_diff>
--- a/03-Hardware/Catalogo-NVIDIA-IA-local.xlsx
+++ b/03-Hardware/Catalogo-NVIDIA-IA-local.xlsx
@@ -10,10 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GPU_Catalogo" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modelo_vs_GPU" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metricas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FP8_vs_FP4" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GPU_Catalogo'!$A$1:$Q$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Metricas'!$A$1:$L$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'FP8_vs_FP4'!$A$1:$D$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3708,4 +3710,273 @@
   <autoFilter ref="A1:L27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>FP8</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>FP4</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Bits por elemento</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Piso elementar; escalas/metadados aumentam a memória real</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Formato típico</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>E4M3/E5M2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>E2M1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FP8 tem mais alcance/precisão; FP4 depende mais de escala</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Modelo denso 8B — pesos elementares (GB)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8B × bits / 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Modelo denso 27B — pesos elementares (GB)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>27</v>
+      </c>
+      <c r="C5" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>27B × bits / 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Modelo denso 70B — pesos elementares (GB)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>70</v>
+      </c>
+      <c r="C6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>70B × bits / 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Uso favorável</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Treinamento misto, serving conservador, pesos/ativações</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Inferência com memória limitada e hardware nativo</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Validar qualidade no modelo real</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Hopper e posteriores, conforme operação</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Blackwell para NVFP4/MXFP4</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Aceleração depende do kernel/runtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FP8 conforme GPU/ROCm</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>HIP documenta FP4 nativo em CDNA4; não em RDNA2/3/4 na tabela consultada</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Não inferir aceleração em Radeon de consumo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MLX/Metal conforme implementação</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Não assumir NVFP4/MXFP4; registrar formato suportado pelo MLX/runtime</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Memória unificada não implica suporte ao tipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Métrica exigida</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tokens/s, TTFT, P50/P95, qualidade</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>tokens/s, TTFT, P50/P95, qualidade</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sem benchmark homogêneo, comparar apenas suporte e memória</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Fontes</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NVIDIA Transformer Engine</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NVIDIA NVFP4; AMD HIP FP4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>[[05-Memoria-e-Performance/Comparativo-FP8-vs-FP4]]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>